<commit_message>
Clean up GV wearables workflow and update consensus
</commit_message>
<xml_diff>
--- a/01_input/00_Manual_input/02_Consensus_frames_template.xlsx
+++ b/01_input/00_Manual_input/02_Consensus_frames_template.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\luxnt\Retail\AAA_Retail\Demand Management GV\10. Automatizzazione file consensus\01_input\00_Manual_input\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8DEDE9E0-1967-4710-ADC6-4A257EF3B87C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5D1D1309-ED70-4868-82F2-94E8CABAC85F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-16320" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-105" yWindow="-16200" windowWidth="14610" windowHeight="15585" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Consensus Frames" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="70" uniqueCount="60">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="74" uniqueCount="61">
   <si>
     <t>year_bucket</t>
   </si>
@@ -105,9 +105,6 @@
   </si>
   <si>
     <t>Forecast Sales da minimo pcs</t>
-  </si>
-  <si>
-    <t>Forecast sales da minmo (last approved)</t>
   </si>
   <si>
     <t>Forecast Sales Tot (pcs)</t>
@@ -234,6 +231,12 @@
   <si>
     <t>Weekly Sales CY</t>
   </si>
+  <si>
+    <t>Volume Error %</t>
+  </si>
+  <si>
+    <t>Forecast  Weekly Sales Tot (pcs)</t>
+  </si>
 </sst>
 </file>
 
@@ -243,7 +246,7 @@
     <numFmt numFmtId="43" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
     <numFmt numFmtId="164" formatCode="_-* #,##0_-;\-* #,##0_-;_-* &quot;-&quot;??_-;_-@_-"/>
   </numFmts>
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="8" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -281,8 +284,23 @@
       <name val="Calibri"/>
       <family val="2"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <i/>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
   </fonts>
-  <fills count="19">
+  <fills count="21">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -378,8 +396,19 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="gray0625">
+        <bgColor theme="7" tint="0.59999389629810485"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="40">
+  <borders count="45">
     <border>
       <left/>
       <right/>
@@ -643,19 +672,6 @@
       <diagonal/>
     </border>
     <border>
-      <left style="double">
-        <color rgb="FF000000"/>
-      </left>
-      <right/>
-      <top style="medium">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom style="medium">
-        <color rgb="FF000000"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
       <left style="medium">
         <color rgb="FF000000"/>
       </left>
@@ -903,6 +919,80 @@
       </left>
       <right style="mediumDashDot">
         <color rgb="FFEDB913"/>
+      </right>
+      <top style="medium">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="mediumDashDot">
+        <color rgb="FFFFC000"/>
+      </left>
+      <right style="mediumDashDot">
+        <color rgb="FFFFC000"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="mediumDashDot">
+        <color rgb="FFFFC000"/>
       </right>
       <top style="medium">
         <color rgb="FF000000"/>
@@ -920,7 +1010,7 @@
     <xf numFmtId="43" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="165">
+  <cellXfs count="177">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -948,16 +1038,15 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="25" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="24" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -969,61 +1058,45 @@
     <xf numFmtId="0" fontId="1" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="164" fontId="0" fillId="8" borderId="24" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="0" fillId="8" borderId="23" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="0" fillId="8" borderId="9" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="0" fillId="8" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="9" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="16" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="10" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="24" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="23" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="26" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="0" fillId="8" borderId="22" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="25" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="0" fillId="8" borderId="21" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="0" fillId="8" borderId="7" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="0" fillId="8" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="7" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="17" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="8" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="22" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="21" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="7" xfId="2" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="17" xfId="2" applyFont="1" applyBorder="1"/>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="13" xfId="2" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="22" xfId="2" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="21" xfId="2" applyFont="1" applyBorder="1"/>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="1" xfId="2" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="9" fontId="1" fillId="9" borderId="24" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="1" fillId="9" borderId="7" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="1" fillId="9" borderId="1" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="1" fillId="6" borderId="7" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="1" fillId="6" borderId="16" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="1" fillId="10" borderId="22" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="1" fillId="10" borderId="21" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="164" fontId="1" fillId="10" borderId="7" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1038,7 +1111,7 @@
     <xf numFmtId="164" fontId="1" fillId="7" borderId="17" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="1" fillId="11" borderId="21" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="1" fillId="11" borderId="20" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="164" fontId="1" fillId="11" borderId="6" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1054,15 +1127,15 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="13" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="29" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="28" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="28" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="29" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="30" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1078,13 +1151,13 @@
     <xf numFmtId="9" fontId="1" fillId="2" borderId="9" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="9" fontId="1" fillId="12" borderId="33" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="1" fillId="2" borderId="30" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="2" fillId="8" borderId="24" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="9" fontId="1" fillId="12" borderId="32" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="1" fillId="2" borderId="29" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="2" fillId="8" borderId="23" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="164" fontId="2" fillId="8" borderId="9" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1102,13 +1175,13 @@
     <xf numFmtId="164" fontId="2" fillId="0" borderId="15" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="2" fillId="0" borderId="24" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="23" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="164" fontId="2" fillId="0" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="2" fillId="8" borderId="22" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="2" fillId="8" borderId="21" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="164" fontId="2" fillId="8" borderId="7" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1126,13 +1199,13 @@
     <xf numFmtId="164" fontId="2" fillId="0" borderId="13" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="2" fillId="0" borderId="22" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="21" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="164" fontId="2" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="2" fillId="8" borderId="21" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="2" fillId="8" borderId="20" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="164" fontId="2" fillId="8" borderId="6" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1147,34 +1220,31 @@
     <xf numFmtId="164" fontId="2" fillId="0" borderId="14" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="2" fillId="0" borderId="21" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="20" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="164" fontId="2" fillId="0" borderId="11" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="2" fillId="0" borderId="31" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="28" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="30" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="27" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="20" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="37" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="36" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="27" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="26" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="1" fillId="9" borderId="22" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="1" fillId="9" borderId="21" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="164" fontId="1" fillId="9" borderId="7" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1189,36 +1259,24 @@
     <xf numFmtId="164" fontId="1" fillId="6" borderId="17" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="8" borderId="38" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="0" fillId="8" borderId="26" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="9" fontId="0" fillId="8" borderId="24" xfId="2" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="0" fillId="8" borderId="37" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="0" fillId="8" borderId="25" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="9" fontId="0" fillId="8" borderId="23" xfId="2" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="9" fontId="0" fillId="8" borderId="5" xfId="2" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="9" xfId="2" applyFont="1" applyBorder="1"/>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="16" xfId="2" applyFont="1" applyBorder="1"/>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="15" xfId="2" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="24" xfId="2" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="23" xfId="2" applyFont="1" applyBorder="1"/>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="5" xfId="2" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="26" xfId="2" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="9" fontId="0" fillId="8" borderId="22" xfId="2" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="25" xfId="2" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="9" fontId="0" fillId="8" borderId="21" xfId="2" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="9" fontId="0" fillId="8" borderId="1" xfId="2" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="32" xfId="2" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="31" xfId="2" applyFont="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="0" fillId="13" borderId="17" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="2" fillId="13" borderId="18" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="5" fillId="6" borderId="13" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="5" fillId="6" borderId="24" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="5" fillId="6" borderId="1" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="164" fontId="5" fillId="7" borderId="13" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="7" borderId="22" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="5" fillId="7" borderId="21" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="164" fontId="5" fillId="7" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1227,79 +1285,125 @@
     <xf numFmtId="164" fontId="5" fillId="5" borderId="14" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="5" borderId="21" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="5" fillId="5" borderId="20" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="164" fontId="5" fillId="5" borderId="11" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="9" fontId="5" fillId="2" borderId="33" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="5" fillId="2" borderId="32" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="9" fontId="5" fillId="2" borderId="34" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="9" fontId="5" fillId="2" borderId="33" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="9" fontId="5" fillId="2" borderId="35" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="9" fontId="5" fillId="2" borderId="36" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="164" fontId="5" fillId="6" borderId="13" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="6" borderId="22" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="5" fillId="6" borderId="21" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="164" fontId="5" fillId="6" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="6" borderId="32" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="7" borderId="32" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="5" borderId="31" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
+    <xf numFmtId="164" fontId="5" fillId="6" borderId="31" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="7" borderId="31" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="5" borderId="30" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="14" borderId="23" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="0" fillId="14" borderId="21" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="2" fillId="14" borderId="23" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="2" fillId="14" borderId="21" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="2" fillId="14" borderId="20" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="38" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="19" borderId="39" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="1" fillId="20" borderId="40" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="1" fillId="20" borderId="39" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="1" fillId="20" borderId="41" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="1" fillId="19" borderId="39" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="1" fillId="19" borderId="42" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="5" fillId="19" borderId="43" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="5" fillId="19" borderId="40" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="5" fillId="19" borderId="41" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="13" borderId="18" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="13" borderId="17" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="9" fontId="6" fillId="0" borderId="17" xfId="2" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="17" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="14" borderId="28" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="3" fillId="14" borderId="23" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="3" fillId="14" borderId="21" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="9" fontId="3" fillId="14" borderId="23" xfId="2" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="9" fontId="3" fillId="14" borderId="21" xfId="2" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="14" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="3" fillId="14" borderId="37" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="5" fillId="16" borderId="21" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="17" borderId="20" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="14" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="9" fontId="5" fillId="18" borderId="32" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="15" borderId="21" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="44" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="164" fontId="0" fillId="14" borderId="24" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="0" fillId="14" borderId="22" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="14" borderId="29" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="9" fontId="0" fillId="14" borderId="24" xfId="2" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="9" fontId="0" fillId="14" borderId="22" xfId="2" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="14" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="0" fillId="14" borderId="38" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="9" fontId="1" fillId="15" borderId="24" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="1" fillId="16" borderId="22" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="1" fillId="17" borderId="21" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="14" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="164" fontId="2" fillId="14" borderId="24" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="2" fillId="14" borderId="22" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="2" fillId="14" borderId="21" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="1" fillId="18" borderId="33" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="1" fillId="15" borderId="22" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="39" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="24" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="9" fontId="2" fillId="0" borderId="1" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="8" borderId="37" xfId="2" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="9" fontId="0" fillId="8" borderId="25" xfId="2" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="9" fontId="3" fillId="14" borderId="37" xfId="2" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="24" xfId="2" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="2" applyFont="1"/>
+    <xf numFmtId="3" fontId="5" fillId="6" borderId="13" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1608,7 +1712,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:O40"/>
+  <dimension ref="A1:O45"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="46.36328125" bestFit="1" customWidth="1"/>
@@ -1616,22 +1720,22 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:15" ht="24" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="146" t="s">
-        <v>55</v>
-      </c>
-      <c r="B1" s="147"/>
-      <c r="C1" s="147"/>
-      <c r="D1" s="147"/>
-      <c r="E1" s="147"/>
-      <c r="F1" s="147"/>
-      <c r="G1" s="147"/>
-      <c r="H1" s="147"/>
-      <c r="I1" s="147"/>
-      <c r="J1" s="147"/>
-      <c r="K1" s="147"/>
-      <c r="L1" s="147"/>
-      <c r="M1" s="147"/>
-      <c r="N1" s="147"/>
+      <c r="A1" s="166" t="s">
+        <v>54</v>
+      </c>
+      <c r="B1" s="167"/>
+      <c r="C1" s="167"/>
+      <c r="D1" s="167"/>
+      <c r="E1" s="167"/>
+      <c r="F1" s="167"/>
+      <c r="G1" s="167"/>
+      <c r="H1" s="167"/>
+      <c r="I1" s="167"/>
+      <c r="J1" s="167"/>
+      <c r="K1" s="167"/>
+      <c r="L1" s="167"/>
+      <c r="M1" s="167"/>
+      <c r="N1" s="167"/>
     </row>
     <row r="2" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
@@ -1682,318 +1786,318 @@
         <v>4</v>
       </c>
       <c r="B3" t="s">
+        <v>40</v>
+      </c>
+      <c r="C3" t="s">
         <v>41</v>
       </c>
-      <c r="C3" t="s">
+      <c r="D3" t="s">
         <v>42</v>
       </c>
-      <c r="D3" t="s">
+      <c r="E3" t="s">
         <v>43</v>
       </c>
-      <c r="E3" t="s">
+      <c r="F3" t="s">
         <v>44</v>
       </c>
-      <c r="F3" t="s">
+      <c r="G3" t="s">
         <v>45</v>
       </c>
-      <c r="G3" t="s">
+      <c r="H3" t="s">
         <v>46</v>
       </c>
-      <c r="H3" t="s">
+      <c r="I3" t="s">
         <v>47</v>
       </c>
-      <c r="I3" t="s">
+      <c r="J3" t="s">
         <v>48</v>
       </c>
-      <c r="J3" t="s">
+      <c r="K3" t="s">
         <v>49</v>
       </c>
-      <c r="K3" t="s">
+      <c r="L3" t="s">
         <v>50</v>
       </c>
-      <c r="L3" t="s">
+      <c r="M3" t="s">
         <v>51</v>
       </c>
-      <c r="M3" t="s">
+      <c r="N3" t="s">
         <v>52</v>
       </c>
-      <c r="N3" t="s">
-        <v>53</v>
-      </c>
     </row>
     <row r="4" spans="1:15" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B4" s="23" t="s">
+      <c r="B4" s="22" t="s">
+        <v>27</v>
+      </c>
+      <c r="C4" s="13" t="s">
         <v>28</v>
       </c>
-      <c r="C4" s="14" t="s">
+      <c r="D4" s="14" t="s">
         <v>29</v>
       </c>
-      <c r="D4" s="15" t="s">
+      <c r="E4" s="15" t="s">
         <v>30</v>
       </c>
-      <c r="E4" s="16" t="s">
+      <c r="F4" s="16" t="s">
         <v>31</v>
       </c>
-      <c r="F4" s="17" t="s">
+      <c r="G4" s="139" t="s">
         <v>32</v>
       </c>
-      <c r="G4" s="164" t="s">
+      <c r="H4" s="17" t="s">
         <v>33</v>
       </c>
-      <c r="H4" s="18" t="s">
+      <c r="I4" s="18" t="s">
         <v>34</v>
       </c>
-      <c r="I4" s="19" t="s">
+      <c r="J4" s="19" t="s">
         <v>35</v>
       </c>
-      <c r="J4" s="20" t="s">
+      <c r="K4" s="20" t="s">
         <v>36</v>
       </c>
-      <c r="K4" s="21" t="s">
+      <c r="L4" s="21" t="s">
         <v>37</v>
       </c>
-      <c r="L4" s="22" t="s">
+      <c r="M4" s="22" t="s">
         <v>38</v>
       </c>
-      <c r="M4" s="23" t="s">
+      <c r="N4" s="23" t="s">
         <v>39</v>
       </c>
-      <c r="N4" s="24" t="s">
-        <v>40</v>
-      </c>
-      <c r="O4" s="13"/>
+      <c r="O4" s="12"/>
     </row>
     <row r="5" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A5" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="B5" s="27"/>
-      <c r="C5" s="28"/>
-      <c r="D5" s="27"/>
-      <c r="E5" s="29"/>
-      <c r="F5" s="30"/>
-      <c r="G5" s="148"/>
-      <c r="H5" s="31"/>
-      <c r="I5" s="32"/>
-      <c r="J5" s="33"/>
-      <c r="K5" s="34"/>
-      <c r="L5" s="34"/>
-      <c r="M5" s="33"/>
-      <c r="N5" s="35"/>
-      <c r="O5" s="13"/>
+      <c r="B5" s="26"/>
+      <c r="C5" s="27"/>
+      <c r="D5" s="26"/>
+      <c r="E5" s="28"/>
+      <c r="F5" s="29"/>
+      <c r="G5" s="134"/>
+      <c r="H5" s="30"/>
+      <c r="I5" s="31"/>
+      <c r="J5" s="32"/>
+      <c r="K5" s="33"/>
+      <c r="L5" s="33"/>
+      <c r="M5" s="32"/>
+      <c r="N5" s="34"/>
+      <c r="O5" s="12"/>
     </row>
     <row r="6" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A6" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="B6" s="36"/>
-      <c r="C6" s="37"/>
-      <c r="D6" s="36"/>
-      <c r="E6" s="38"/>
-      <c r="F6" s="39"/>
-      <c r="G6" s="149"/>
-      <c r="H6" s="40"/>
-      <c r="I6" s="41"/>
-      <c r="J6" s="42"/>
-      <c r="K6" s="43"/>
-      <c r="L6" s="43"/>
-      <c r="M6" s="42"/>
-      <c r="N6" s="39"/>
-      <c r="O6" s="13"/>
+      <c r="B6" s="35"/>
+      <c r="C6" s="36"/>
+      <c r="D6" s="35"/>
+      <c r="E6" s="37"/>
+      <c r="F6" s="38"/>
+      <c r="G6" s="135"/>
+      <c r="H6" s="39"/>
+      <c r="I6" s="40"/>
+      <c r="J6" s="41"/>
+      <c r="K6" s="42"/>
+      <c r="L6" s="42"/>
+      <c r="M6" s="41"/>
+      <c r="N6" s="38"/>
+      <c r="O6" s="12"/>
     </row>
     <row r="7" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A7" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="B7" s="36"/>
-      <c r="C7" s="37"/>
-      <c r="D7" s="36"/>
-      <c r="E7" s="38"/>
-      <c r="F7" s="39"/>
-      <c r="G7" s="149"/>
-      <c r="H7" s="40"/>
-      <c r="I7" s="41"/>
-      <c r="J7" s="42"/>
-      <c r="K7" s="43"/>
-      <c r="L7" s="43"/>
-      <c r="M7" s="42"/>
-      <c r="N7" s="39"/>
-      <c r="O7" s="13"/>
+      <c r="B7" s="35"/>
+      <c r="C7" s="36"/>
+      <c r="D7" s="35"/>
+      <c r="E7" s="37"/>
+      <c r="F7" s="38"/>
+      <c r="G7" s="135"/>
+      <c r="H7" s="39"/>
+      <c r="I7" s="40"/>
+      <c r="J7" s="41"/>
+      <c r="K7" s="42"/>
+      <c r="L7" s="42"/>
+      <c r="M7" s="41"/>
+      <c r="N7" s="38"/>
+      <c r="O7" s="12"/>
     </row>
     <row r="8" spans="1:15" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A8" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="B8" s="36"/>
-      <c r="C8" s="37"/>
-      <c r="D8" s="36"/>
-      <c r="E8" s="38"/>
-      <c r="F8" s="39"/>
-      <c r="G8" s="149"/>
-      <c r="H8" s="125"/>
-      <c r="I8" s="41"/>
-      <c r="J8" s="42"/>
-      <c r="K8" s="43"/>
-      <c r="L8" s="43"/>
-      <c r="M8" s="42"/>
-      <c r="N8" s="39"/>
-      <c r="O8" s="13"/>
+      <c r="B8" s="35"/>
+      <c r="C8" s="36"/>
+      <c r="D8" s="35"/>
+      <c r="E8" s="37"/>
+      <c r="F8" s="38"/>
+      <c r="G8" s="135"/>
+      <c r="H8" s="117"/>
+      <c r="I8" s="40"/>
+      <c r="J8" s="41"/>
+      <c r="K8" s="42"/>
+      <c r="L8" s="42"/>
+      <c r="M8" s="41"/>
+      <c r="N8" s="38"/>
+      <c r="O8" s="12"/>
     </row>
     <row r="9" spans="1:15" ht="35" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A9" s="66"/>
-      <c r="B9" s="67"/>
-      <c r="C9" s="67"/>
-      <c r="D9" s="67"/>
-      <c r="E9" s="67"/>
-      <c r="F9" s="68"/>
-      <c r="G9" s="150"/>
-      <c r="H9" s="69"/>
-      <c r="I9" s="68"/>
-      <c r="J9" s="68"/>
-      <c r="K9" s="68"/>
-      <c r="L9" s="68"/>
-      <c r="M9" s="68"/>
+      <c r="A9" s="59"/>
+      <c r="B9" s="60"/>
+      <c r="C9" s="60"/>
+      <c r="D9" s="60"/>
+      <c r="E9" s="60"/>
+      <c r="F9" s="61"/>
+      <c r="G9" s="153"/>
+      <c r="H9" s="62"/>
+      <c r="I9" s="61"/>
+      <c r="J9" s="61"/>
+      <c r="K9" s="61"/>
+      <c r="L9" s="61"/>
+      <c r="M9" s="61"/>
       <c r="N9" s="4"/>
     </row>
     <row r="10" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A10" s="6" t="s">
-        <v>56</v>
-      </c>
-      <c r="B10" s="27"/>
-      <c r="C10" s="28"/>
-      <c r="D10" s="27"/>
-      <c r="E10" s="29"/>
-      <c r="F10" s="30"/>
-      <c r="G10" s="148"/>
-      <c r="H10" s="31"/>
-      <c r="I10" s="32"/>
-      <c r="J10" s="33"/>
-      <c r="K10" s="34"/>
-      <c r="L10" s="34"/>
-      <c r="M10" s="33"/>
-      <c r="N10" s="35"/>
-      <c r="O10" s="13"/>
+        <v>55</v>
+      </c>
+      <c r="B10" s="26"/>
+      <c r="C10" s="27"/>
+      <c r="D10" s="26"/>
+      <c r="E10" s="28"/>
+      <c r="F10" s="29"/>
+      <c r="G10" s="154"/>
+      <c r="H10" s="30"/>
+      <c r="I10" s="31"/>
+      <c r="J10" s="32"/>
+      <c r="K10" s="33"/>
+      <c r="L10" s="33"/>
+      <c r="M10" s="32"/>
+      <c r="N10" s="34"/>
+      <c r="O10" s="12"/>
     </row>
     <row r="11" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A11" s="2" t="s">
-        <v>57</v>
-      </c>
-      <c r="B11" s="36"/>
-      <c r="C11" s="37"/>
-      <c r="D11" s="36"/>
-      <c r="E11" s="38"/>
-      <c r="F11" s="39"/>
-      <c r="G11" s="149"/>
-      <c r="H11" s="40"/>
-      <c r="I11" s="41"/>
-      <c r="J11" s="42"/>
-      <c r="K11" s="43"/>
-      <c r="L11" s="43"/>
-      <c r="M11" s="42"/>
-      <c r="N11" s="39"/>
-      <c r="O11" s="13"/>
+        <v>56</v>
+      </c>
+      <c r="B11" s="35"/>
+      <c r="C11" s="36"/>
+      <c r="D11" s="35"/>
+      <c r="E11" s="37"/>
+      <c r="F11" s="38"/>
+      <c r="G11" s="155"/>
+      <c r="H11" s="39"/>
+      <c r="I11" s="40"/>
+      <c r="J11" s="41"/>
+      <c r="K11" s="42"/>
+      <c r="L11" s="42"/>
+      <c r="M11" s="41"/>
+      <c r="N11" s="38"/>
+      <c r="O11" s="12"/>
     </row>
     <row r="12" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A12" s="2" t="s">
-        <v>58</v>
-      </c>
-      <c r="B12" s="36"/>
-      <c r="C12" s="37"/>
-      <c r="D12" s="36"/>
-      <c r="E12" s="38"/>
-      <c r="F12" s="39"/>
-      <c r="G12" s="149"/>
-      <c r="H12" s="40"/>
-      <c r="I12" s="41"/>
-      <c r="J12" s="42"/>
-      <c r="K12" s="43"/>
-      <c r="L12" s="43"/>
-      <c r="M12" s="42"/>
-      <c r="N12" s="39"/>
-      <c r="O12" s="13"/>
+        <v>57</v>
+      </c>
+      <c r="B12" s="35"/>
+      <c r="C12" s="36"/>
+      <c r="D12" s="35"/>
+      <c r="E12" s="37"/>
+      <c r="F12" s="38"/>
+      <c r="G12" s="155"/>
+      <c r="H12" s="39"/>
+      <c r="I12" s="40"/>
+      <c r="J12" s="41"/>
+      <c r="K12" s="42"/>
+      <c r="L12" s="42"/>
+      <c r="M12" s="41"/>
+      <c r="N12" s="38"/>
+      <c r="O12" s="12"/>
     </row>
     <row r="13" spans="1:15" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A13" s="2" t="s">
-        <v>59</v>
-      </c>
-      <c r="B13" s="36"/>
-      <c r="C13" s="37"/>
-      <c r="D13" s="36"/>
-      <c r="E13" s="38"/>
-      <c r="F13" s="39"/>
-      <c r="G13" s="149"/>
-      <c r="H13" s="125"/>
-      <c r="I13" s="41"/>
-      <c r="J13" s="42"/>
-      <c r="K13" s="43"/>
-      <c r="L13" s="43"/>
-      <c r="M13" s="42"/>
-      <c r="N13" s="39"/>
-      <c r="O13" s="13"/>
+        <v>58</v>
+      </c>
+      <c r="B13" s="35"/>
+      <c r="C13" s="36"/>
+      <c r="D13" s="35"/>
+      <c r="E13" s="37"/>
+      <c r="F13" s="38"/>
+      <c r="G13" s="155"/>
+      <c r="H13" s="150"/>
+      <c r="I13" s="40"/>
+      <c r="J13" s="41"/>
+      <c r="K13" s="42"/>
+      <c r="L13" s="42"/>
+      <c r="M13" s="41"/>
+      <c r="N13" s="38"/>
+      <c r="O13" s="12"/>
     </row>
     <row r="14" spans="1:15" ht="35" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A14" s="66"/>
-      <c r="B14" s="67"/>
-      <c r="C14" s="67"/>
-      <c r="D14" s="67"/>
-      <c r="E14" s="67"/>
-      <c r="F14" s="68"/>
-      <c r="G14" s="150"/>
-      <c r="H14" s="69"/>
-      <c r="I14" s="68"/>
-      <c r="J14" s="68"/>
-      <c r="K14" s="68"/>
-      <c r="L14" s="68"/>
-      <c r="M14" s="68"/>
+      <c r="A14" s="59"/>
+      <c r="B14" s="60"/>
+      <c r="C14" s="60"/>
+      <c r="D14" s="60"/>
+      <c r="E14" s="60"/>
+      <c r="F14" s="61"/>
+      <c r="G14" s="153"/>
+      <c r="H14" s="62"/>
+      <c r="I14" s="61"/>
+      <c r="J14" s="61"/>
+      <c r="K14" s="61"/>
+      <c r="L14" s="61"/>
+      <c r="M14" s="61"/>
       <c r="N14" s="4"/>
     </row>
     <row r="15" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A15" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="B15" s="114"/>
-      <c r="C15" s="115"/>
-      <c r="D15" s="114"/>
-      <c r="E15" s="115"/>
-      <c r="F15" s="116"/>
-      <c r="G15" s="151"/>
-      <c r="H15" s="117"/>
-      <c r="I15" s="118"/>
-      <c r="J15" s="119"/>
-      <c r="K15" s="120"/>
-      <c r="L15" s="120"/>
-      <c r="M15" s="119"/>
-      <c r="N15" s="121"/>
-      <c r="O15" s="13"/>
+      <c r="B15" s="106"/>
+      <c r="C15" s="107"/>
+      <c r="D15" s="106"/>
+      <c r="E15" s="107"/>
+      <c r="F15" s="108"/>
+      <c r="G15" s="156"/>
+      <c r="H15" s="109"/>
+      <c r="I15" s="110"/>
+      <c r="J15" s="111"/>
+      <c r="K15" s="112"/>
+      <c r="L15" s="112"/>
+      <c r="M15" s="111"/>
+      <c r="N15" s="113"/>
+      <c r="O15" s="12"/>
     </row>
     <row r="16" spans="1:15" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A16" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="B16" s="122"/>
-      <c r="C16" s="123"/>
-      <c r="D16" s="122"/>
-      <c r="E16" s="123"/>
-      <c r="F16" s="44"/>
-      <c r="G16" s="152"/>
-      <c r="H16" s="45"/>
-      <c r="I16" s="46"/>
-      <c r="J16" s="47"/>
-      <c r="K16" s="48"/>
-      <c r="L16" s="48"/>
-      <c r="M16" s="47"/>
-      <c r="N16" s="124"/>
-      <c r="O16" s="13"/>
+      <c r="B16" s="114"/>
+      <c r="C16" s="115"/>
+      <c r="D16" s="114"/>
+      <c r="E16" s="115"/>
+      <c r="F16" s="43"/>
+      <c r="G16" s="157"/>
+      <c r="H16" s="150"/>
+      <c r="I16" s="44"/>
+      <c r="J16" s="45"/>
+      <c r="K16" s="46"/>
+      <c r="L16" s="46"/>
+      <c r="M16" s="45"/>
+      <c r="N16" s="116"/>
+      <c r="O16" s="12"/>
     </row>
     <row r="17" spans="1:15" ht="35" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A17" s="3"/>
-      <c r="B17" s="25"/>
-      <c r="C17" s="25"/>
-      <c r="D17" s="25"/>
-      <c r="E17" s="25"/>
+      <c r="B17" s="24"/>
+      <c r="C17" s="24"/>
+      <c r="D17" s="24"/>
+      <c r="E17" s="24"/>
       <c r="F17" s="4"/>
-      <c r="G17" s="153"/>
-      <c r="H17" s="12"/>
+      <c r="G17" s="158"/>
+      <c r="H17" s="11"/>
       <c r="I17" s="4"/>
       <c r="J17" s="4"/>
       <c r="K17" s="4"/>
@@ -2005,49 +2109,49 @@
       <c r="A18" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="B18" s="112"/>
-      <c r="C18" s="113"/>
-      <c r="D18" s="112"/>
-      <c r="E18" s="29"/>
-      <c r="F18" s="39"/>
-      <c r="G18" s="154"/>
-      <c r="H18" s="45"/>
-      <c r="I18" s="46"/>
-      <c r="J18" s="47"/>
-      <c r="K18" s="48"/>
-      <c r="L18" s="48"/>
-      <c r="M18" s="47"/>
-      <c r="N18" s="48"/>
-      <c r="O18" s="13"/>
+      <c r="B18" s="104"/>
+      <c r="C18" s="105"/>
+      <c r="D18" s="104"/>
+      <c r="E18" s="28"/>
+      <c r="F18" s="38"/>
+      <c r="G18" s="159"/>
+      <c r="H18" s="151"/>
+      <c r="I18" s="44"/>
+      <c r="J18" s="45"/>
+      <c r="K18" s="46"/>
+      <c r="L18" s="46"/>
+      <c r="M18" s="45"/>
+      <c r="N18" s="46"/>
+      <c r="O18" s="12"/>
     </row>
     <row r="19" spans="1:15" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A19" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="B19" s="36"/>
-      <c r="C19" s="38"/>
-      <c r="D19" s="112"/>
-      <c r="E19" s="38"/>
-      <c r="F19" s="39"/>
-      <c r="G19" s="154"/>
-      <c r="H19" s="40"/>
-      <c r="I19" s="64"/>
-      <c r="J19" s="42"/>
-      <c r="K19" s="43"/>
-      <c r="L19" s="43"/>
-      <c r="M19" s="42"/>
-      <c r="N19" s="43"/>
-      <c r="O19" s="13"/>
+      <c r="B19" s="35"/>
+      <c r="C19" s="37"/>
+      <c r="D19" s="104"/>
+      <c r="E19" s="37"/>
+      <c r="F19" s="38"/>
+      <c r="G19" s="159"/>
+      <c r="H19" s="152"/>
+      <c r="I19" s="57"/>
+      <c r="J19" s="41"/>
+      <c r="K19" s="42"/>
+      <c r="L19" s="42"/>
+      <c r="M19" s="41"/>
+      <c r="N19" s="42"/>
+      <c r="O19" s="12"/>
     </row>
     <row r="20" spans="1:15" ht="35" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A20" s="3"/>
-      <c r="B20" s="25"/>
-      <c r="C20" s="25"/>
-      <c r="D20" s="25"/>
-      <c r="E20" s="25"/>
+      <c r="B20" s="24"/>
+      <c r="C20" s="24"/>
+      <c r="D20" s="24"/>
+      <c r="E20" s="24"/>
       <c r="F20" s="4"/>
-      <c r="G20" s="153"/>
-      <c r="H20" s="12"/>
+      <c r="G20" s="158"/>
+      <c r="H20" s="11"/>
       <c r="I20" s="4"/>
       <c r="J20" s="4"/>
       <c r="K20" s="4"/>
@@ -2056,312 +2160,328 @@
       <c r="N20" s="4"/>
     </row>
     <row r="21" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A21" s="7" t="s">
+      <c r="A21" s="64" t="s">
+        <v>25</v>
+      </c>
+      <c r="B21" s="68"/>
+      <c r="C21" s="65"/>
+      <c r="D21" s="68"/>
+      <c r="E21" s="66"/>
+      <c r="F21" s="67"/>
+      <c r="G21" s="163"/>
+      <c r="H21" s="69"/>
+      <c r="I21" s="124"/>
+      <c r="J21" s="125"/>
+      <c r="K21" s="126"/>
+      <c r="L21" s="126"/>
+      <c r="M21" s="125"/>
+      <c r="N21" s="127"/>
+      <c r="O21" s="12"/>
+    </row>
+    <row r="22" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A22" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="B22" s="99"/>
+      <c r="C22" s="100"/>
+      <c r="D22" s="99"/>
+      <c r="E22" s="101"/>
+      <c r="F22" s="102"/>
+      <c r="G22" s="164"/>
+      <c r="H22" s="103"/>
+      <c r="I22" s="128"/>
+      <c r="J22" s="129"/>
+      <c r="K22" s="130"/>
+      <c r="L22" s="130"/>
+      <c r="M22" s="129"/>
+      <c r="N22" s="131"/>
+      <c r="O22" s="12"/>
+    </row>
+    <row r="23" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A23" s="8" t="s">
+        <v>60</v>
+      </c>
+      <c r="B23" s="47"/>
+      <c r="C23" s="48"/>
+      <c r="D23" s="47"/>
+      <c r="E23" s="49"/>
+      <c r="F23" s="50"/>
+      <c r="G23" s="160"/>
+      <c r="H23" s="51"/>
+      <c r="I23" s="118"/>
+      <c r="J23" s="119"/>
+      <c r="K23" s="120"/>
+      <c r="L23" s="120"/>
+      <c r="M23" s="119"/>
+      <c r="N23" s="132"/>
+      <c r="O23" s="12"/>
+    </row>
+    <row r="24" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A24" s="140" t="s">
+        <v>59</v>
+      </c>
+      <c r="B24" s="141"/>
+      <c r="C24" s="142"/>
+      <c r="D24" s="141"/>
+      <c r="E24" s="143"/>
+      <c r="F24" s="144"/>
+      <c r="G24" s="147"/>
+      <c r="H24" s="145"/>
+      <c r="I24" s="146"/>
+      <c r="J24" s="147"/>
+      <c r="K24" s="148"/>
+      <c r="L24" s="148"/>
+      <c r="M24" s="147"/>
+      <c r="N24" s="148"/>
+      <c r="O24" s="12"/>
+    </row>
+    <row r="25" spans="1:15" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A25" s="9" t="s">
         <v>26</v>
       </c>
-      <c r="B21" s="49"/>
-      <c r="C21" s="50"/>
-      <c r="D21" s="49"/>
-      <c r="E21" s="51"/>
-      <c r="F21" s="52"/>
-      <c r="G21" s="155"/>
-      <c r="H21" s="53"/>
-      <c r="I21" s="127"/>
-      <c r="J21" s="128"/>
-      <c r="K21" s="129"/>
-      <c r="L21" s="129"/>
-      <c r="M21" s="128"/>
-      <c r="N21" s="129"/>
-      <c r="O21" s="13"/>
-    </row>
-    <row r="22" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A22" s="8" t="s">
-        <v>25</v>
-      </c>
-      <c r="B22" s="54"/>
-      <c r="C22" s="55"/>
-      <c r="D22" s="54"/>
-      <c r="E22" s="56"/>
-      <c r="F22" s="57"/>
-      <c r="G22" s="156"/>
-      <c r="H22" s="58"/>
-      <c r="I22" s="130"/>
-      <c r="J22" s="131"/>
-      <c r="K22" s="132"/>
-      <c r="L22" s="132"/>
-      <c r="M22" s="131"/>
-      <c r="N22" s="132"/>
-      <c r="O22" s="13"/>
-    </row>
-    <row r="23" spans="1:15" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A23" s="9" t="s">
-        <v>27</v>
-      </c>
-      <c r="B23" s="59"/>
-      <c r="C23" s="60"/>
-      <c r="D23" s="59"/>
-      <c r="E23" s="61"/>
-      <c r="F23" s="62"/>
-      <c r="G23" s="157"/>
-      <c r="H23" s="63"/>
-      <c r="I23" s="133"/>
-      <c r="J23" s="134"/>
-      <c r="K23" s="135"/>
-      <c r="L23" s="135"/>
-      <c r="M23" s="134"/>
-      <c r="N23" s="135"/>
-      <c r="O23" s="13"/>
-    </row>
-    <row r="24" spans="1:15" ht="35" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A24" s="5"/>
-      <c r="B24" s="26"/>
-      <c r="C24" s="26"/>
-      <c r="D24" s="26"/>
-      <c r="E24" s="26"/>
-      <c r="G24" s="158"/>
-      <c r="H24" s="10"/>
-    </row>
-    <row r="25" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A25" s="6" t="s">
+      <c r="B25" s="52"/>
+      <c r="C25" s="53"/>
+      <c r="D25" s="52"/>
+      <c r="E25" s="54"/>
+      <c r="F25" s="55"/>
+      <c r="G25" s="161"/>
+      <c r="H25" s="56"/>
+      <c r="I25" s="121"/>
+      <c r="J25" s="122"/>
+      <c r="K25" s="123"/>
+      <c r="L25" s="123"/>
+      <c r="M25" s="122"/>
+      <c r="N25" s="133"/>
+      <c r="O25" s="12"/>
+    </row>
+    <row r="26" spans="1:15" ht="35" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A26" s="5"/>
+      <c r="B26" s="25"/>
+      <c r="C26" s="25"/>
+      <c r="D26" s="25"/>
+      <c r="E26" s="25"/>
+      <c r="G26" s="162"/>
+      <c r="H26" s="10"/>
+    </row>
+    <row r="27" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A27" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="B25" s="77"/>
-      <c r="C25" s="78"/>
-      <c r="D25" s="77"/>
-      <c r="E25" s="79"/>
-      <c r="F25" s="80"/>
-      <c r="G25" s="159"/>
-      <c r="H25" s="81"/>
-      <c r="I25" s="82"/>
-      <c r="J25" s="83"/>
-      <c r="K25" s="84"/>
-      <c r="L25" s="84"/>
-      <c r="M25" s="83"/>
-      <c r="N25" s="84"/>
-      <c r="O25" s="13"/>
-    </row>
-    <row r="26" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A26" s="2" t="s">
+      <c r="B27" s="70"/>
+      <c r="C27" s="71"/>
+      <c r="D27" s="70"/>
+      <c r="E27" s="72"/>
+      <c r="F27" s="73"/>
+      <c r="G27" s="136"/>
+      <c r="H27" s="74"/>
+      <c r="I27" s="75"/>
+      <c r="J27" s="76"/>
+      <c r="K27" s="77"/>
+      <c r="L27" s="77"/>
+      <c r="M27" s="76"/>
+      <c r="N27" s="77"/>
+      <c r="O27" s="12"/>
+    </row>
+    <row r="28" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A28" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="B26" s="85"/>
-      <c r="C26" s="86"/>
-      <c r="D26" s="85"/>
-      <c r="E26" s="87"/>
-      <c r="F26" s="88"/>
-      <c r="G26" s="160"/>
-      <c r="H26" s="89"/>
-      <c r="I26" s="90"/>
-      <c r="J26" s="91"/>
-      <c r="K26" s="92"/>
-      <c r="L26" s="92"/>
-      <c r="M26" s="91"/>
-      <c r="N26" s="92"/>
-      <c r="O26" s="13"/>
-    </row>
-    <row r="27" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A27" s="2" t="s">
+      <c r="B28" s="78"/>
+      <c r="C28" s="79"/>
+      <c r="D28" s="78"/>
+      <c r="E28" s="80"/>
+      <c r="F28" s="81"/>
+      <c r="G28" s="137"/>
+      <c r="H28" s="82"/>
+      <c r="I28" s="83"/>
+      <c r="J28" s="84"/>
+      <c r="K28" s="85"/>
+      <c r="L28" s="85"/>
+      <c r="M28" s="84"/>
+      <c r="N28" s="85"/>
+      <c r="O28" s="12"/>
+    </row>
+    <row r="29" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A29" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="B27" s="85"/>
-      <c r="C27" s="86"/>
-      <c r="D27" s="85"/>
-      <c r="E27" s="87"/>
-      <c r="F27" s="88"/>
-      <c r="G27" s="160"/>
-      <c r="H27" s="89"/>
-      <c r="I27" s="90"/>
-      <c r="J27" s="91"/>
-      <c r="K27" s="92"/>
-      <c r="L27" s="92"/>
-      <c r="M27" s="91"/>
-      <c r="N27" s="92"/>
-      <c r="O27" s="13"/>
-    </row>
-    <row r="28" spans="1:15" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A28" s="70" t="s">
+      <c r="B29" s="78"/>
+      <c r="C29" s="79"/>
+      <c r="D29" s="78"/>
+      <c r="E29" s="80"/>
+      <c r="F29" s="81"/>
+      <c r="G29" s="137"/>
+      <c r="H29" s="82"/>
+      <c r="I29" s="83"/>
+      <c r="J29" s="84"/>
+      <c r="K29" s="85"/>
+      <c r="L29" s="85"/>
+      <c r="M29" s="84"/>
+      <c r="N29" s="85"/>
+      <c r="O29" s="12"/>
+    </row>
+    <row r="30" spans="1:15" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A30" s="63" t="s">
         <v>16</v>
       </c>
-      <c r="B28" s="93"/>
-      <c r="C28" s="94"/>
-      <c r="D28" s="93"/>
-      <c r="E28" s="95"/>
-      <c r="F28" s="96"/>
-      <c r="G28" s="161"/>
-      <c r="H28" s="126"/>
-      <c r="I28" s="97"/>
-      <c r="J28" s="98"/>
-      <c r="K28" s="99"/>
-      <c r="L28" s="99"/>
-      <c r="M28" s="98"/>
-      <c r="N28" s="100"/>
-      <c r="O28" s="13"/>
-    </row>
-    <row r="29" spans="1:15" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="G29" s="158"/>
-      <c r="H29" s="10"/>
-    </row>
-    <row r="30" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A30" s="6" t="s">
+      <c r="B30" s="86"/>
+      <c r="C30" s="87"/>
+      <c r="D30" s="86"/>
+      <c r="E30" s="88"/>
+      <c r="F30" s="89"/>
+      <c r="G30" s="138"/>
+      <c r="H30" s="149"/>
+      <c r="I30" s="90"/>
+      <c r="J30" s="91"/>
+      <c r="K30" s="92"/>
+      <c r="L30" s="92"/>
+      <c r="M30" s="91"/>
+      <c r="N30" s="93"/>
+      <c r="O30" s="12"/>
+    </row>
+    <row r="31" spans="1:15" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="G31" s="162"/>
+      <c r="H31" s="10"/>
+    </row>
+    <row r="32" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A32" s="6" t="s">
         <v>17</v>
       </c>
-      <c r="B30" s="77"/>
-      <c r="C30" s="78"/>
-      <c r="D30" s="77"/>
-      <c r="E30" s="79"/>
-      <c r="F30" s="80"/>
-      <c r="G30" s="159"/>
-      <c r="H30" s="81"/>
-      <c r="I30" s="82"/>
-      <c r="J30" s="83"/>
-      <c r="K30" s="84"/>
-      <c r="L30" s="84"/>
-      <c r="M30" s="83"/>
-      <c r="N30" s="84"/>
-      <c r="O30" s="13"/>
-    </row>
-    <row r="31" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A31" s="2" t="s">
+      <c r="B32" s="70"/>
+      <c r="C32" s="71"/>
+      <c r="D32" s="70"/>
+      <c r="E32" s="72"/>
+      <c r="F32" s="73"/>
+      <c r="G32" s="136"/>
+      <c r="H32" s="74"/>
+      <c r="I32" s="75"/>
+      <c r="J32" s="76"/>
+      <c r="K32" s="77"/>
+      <c r="L32" s="77"/>
+      <c r="M32" s="76"/>
+      <c r="N32" s="77"/>
+      <c r="O32" s="12"/>
+    </row>
+    <row r="33" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A33" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="B31" s="85"/>
-      <c r="C31" s="86"/>
-      <c r="D31" s="85"/>
-      <c r="E31" s="87"/>
-      <c r="F31" s="88"/>
-      <c r="G31" s="160"/>
-      <c r="H31" s="89"/>
-      <c r="I31" s="90"/>
-      <c r="J31" s="91"/>
-      <c r="K31" s="92"/>
-      <c r="L31" s="92"/>
-      <c r="M31" s="91"/>
-      <c r="N31" s="92"/>
-      <c r="O31" s="13"/>
-    </row>
-    <row r="32" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A32" s="2" t="s">
-        <v>54</v>
-      </c>
-      <c r="B32" s="85"/>
-      <c r="C32" s="86"/>
-      <c r="D32" s="85"/>
-      <c r="E32" s="87"/>
-      <c r="F32" s="88"/>
-      <c r="G32" s="160"/>
-      <c r="H32" s="89"/>
-      <c r="I32" s="90"/>
-      <c r="J32" s="91"/>
-      <c r="K32" s="92"/>
-      <c r="L32" s="92"/>
-      <c r="M32" s="91"/>
-      <c r="N32" s="92"/>
-      <c r="O32" s="13"/>
-    </row>
-    <row r="33" spans="1:15" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A33" s="70" t="s">
+      <c r="B33" s="78"/>
+      <c r="C33" s="79"/>
+      <c r="D33" s="78"/>
+      <c r="E33" s="80"/>
+      <c r="F33" s="81"/>
+      <c r="G33" s="137"/>
+      <c r="H33" s="82"/>
+      <c r="I33" s="83"/>
+      <c r="J33" s="84"/>
+      <c r="K33" s="85"/>
+      <c r="L33" s="85"/>
+      <c r="M33" s="84"/>
+      <c r="N33" s="85"/>
+      <c r="O33" s="12"/>
+    </row>
+    <row r="34" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A34" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="B34" s="78"/>
+      <c r="C34" s="79"/>
+      <c r="D34" s="78"/>
+      <c r="E34" s="80"/>
+      <c r="F34" s="81"/>
+      <c r="G34" s="137"/>
+      <c r="H34" s="82"/>
+      <c r="I34" s="83"/>
+      <c r="J34" s="84"/>
+      <c r="K34" s="85"/>
+      <c r="L34" s="85"/>
+      <c r="M34" s="84"/>
+      <c r="N34" s="85"/>
+      <c r="O34" s="12"/>
+    </row>
+    <row r="35" spans="1:15" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A35" s="63" t="s">
         <v>19</v>
       </c>
-      <c r="B33" s="93"/>
-      <c r="C33" s="94"/>
-      <c r="D33" s="93"/>
-      <c r="E33" s="95"/>
-      <c r="F33" s="96"/>
-      <c r="G33" s="161"/>
-      <c r="H33" s="126"/>
-      <c r="I33" s="97"/>
-      <c r="J33" s="98"/>
-      <c r="K33" s="99"/>
-      <c r="L33" s="99"/>
-      <c r="M33" s="98"/>
-      <c r="N33" s="100"/>
-      <c r="O33" s="13"/>
-    </row>
-    <row r="34" spans="1:15" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="G34" s="158"/>
-      <c r="H34" s="10"/>
-    </row>
-    <row r="35" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A35" s="71" t="s">
-        <v>20</v>
-      </c>
-      <c r="B35" s="75"/>
-      <c r="C35" s="72"/>
-      <c r="D35" s="75"/>
-      <c r="E35" s="73"/>
-      <c r="F35" s="74"/>
-      <c r="G35" s="162"/>
-      <c r="H35" s="76"/>
-      <c r="I35" s="136"/>
-      <c r="J35" s="137"/>
-      <c r="K35" s="138"/>
-      <c r="L35" s="138"/>
-      <c r="M35" s="137"/>
-      <c r="N35" s="139"/>
-    </row>
-    <row r="36" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A36" s="7" t="s">
-        <v>23</v>
-      </c>
-      <c r="B36" s="107"/>
-      <c r="C36" s="108"/>
-      <c r="D36" s="107"/>
-      <c r="E36" s="109"/>
-      <c r="F36" s="110"/>
-      <c r="G36" s="163"/>
-      <c r="H36" s="111"/>
-      <c r="I36" s="140"/>
-      <c r="J36" s="141"/>
-      <c r="K36" s="142"/>
-      <c r="L36" s="142"/>
-      <c r="M36" s="141"/>
-      <c r="N36" s="143"/>
-    </row>
-    <row r="37" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A37" s="8" t="s">
-        <v>24</v>
-      </c>
-      <c r="B37" s="54"/>
-      <c r="C37" s="55"/>
-      <c r="D37" s="54"/>
-      <c r="E37" s="56"/>
-      <c r="F37" s="57"/>
-      <c r="G37" s="156"/>
-      <c r="H37" s="58"/>
-      <c r="I37" s="130"/>
-      <c r="J37" s="131"/>
-      <c r="K37" s="132"/>
-      <c r="L37" s="132"/>
-      <c r="M37" s="131"/>
-      <c r="N37" s="144"/>
-    </row>
-    <row r="38" spans="1:15" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A38" s="9" t="s">
-        <v>7</v>
-      </c>
-      <c r="B38" s="59"/>
-      <c r="C38" s="60"/>
-      <c r="D38" s="59"/>
-      <c r="E38" s="61"/>
-      <c r="F38" s="62"/>
-      <c r="G38" s="157"/>
-      <c r="H38" s="63"/>
-      <c r="I38" s="133"/>
-      <c r="J38" s="134"/>
-      <c r="K38" s="135"/>
-      <c r="L38" s="135"/>
-      <c r="M38" s="134"/>
-      <c r="N38" s="145"/>
+      <c r="B35" s="86"/>
+      <c r="C35" s="87"/>
+      <c r="D35" s="86"/>
+      <c r="E35" s="88"/>
+      <c r="F35" s="89"/>
+      <c r="G35" s="138"/>
+      <c r="H35" s="149"/>
+      <c r="I35" s="90"/>
+      <c r="J35" s="91"/>
+      <c r="K35" s="92"/>
+      <c r="L35" s="92"/>
+      <c r="M35" s="91"/>
+      <c r="N35" s="93"/>
+      <c r="O35" s="12"/>
+    </row>
+    <row r="36" spans="1:15" ht="35" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A36" s="3"/>
+      <c r="B36" s="24"/>
+      <c r="C36" s="24"/>
+      <c r="D36" s="24"/>
+      <c r="E36" s="24"/>
+      <c r="F36" s="4"/>
+      <c r="G36" s="158"/>
+      <c r="H36" s="11"/>
+      <c r="I36" s="4"/>
+      <c r="J36" s="4"/>
+      <c r="K36" s="4"/>
+      <c r="L36" s="4"/>
+      <c r="M36" s="4"/>
+      <c r="N36" s="4"/>
+    </row>
+    <row r="37" spans="1:15" s="175" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A37" s="170" t="s">
+        <v>5</v>
+      </c>
+      <c r="B37" s="171"/>
+      <c r="C37" s="172"/>
+      <c r="D37" s="171"/>
+      <c r="E37" s="107"/>
+      <c r="F37" s="43"/>
+      <c r="G37" s="173"/>
+      <c r="H37" s="151"/>
+      <c r="I37" s="44"/>
+      <c r="J37" s="45"/>
+      <c r="K37" s="46"/>
+      <c r="L37" s="46"/>
+      <c r="M37" s="45"/>
+      <c r="N37" s="46"/>
+      <c r="O37" s="174"/>
+    </row>
+    <row r="38" spans="1:15" s="169" customFormat="1" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A38" s="85" t="s">
+        <v>6</v>
+      </c>
+      <c r="B38" s="35"/>
+      <c r="C38" s="37"/>
+      <c r="D38" s="104"/>
+      <c r="E38" s="37"/>
+      <c r="F38" s="38"/>
+      <c r="G38" s="159"/>
+      <c r="H38" s="152"/>
+      <c r="I38" s="57"/>
+      <c r="J38" s="41"/>
+      <c r="K38" s="42"/>
+      <c r="L38" s="42"/>
+      <c r="M38" s="41"/>
+      <c r="N38" s="42"/>
+      <c r="O38" s="168"/>
     </row>
     <row r="39" spans="1:15" ht="35" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A39" s="3"/>
-      <c r="B39" s="4"/>
-      <c r="C39" s="4"/>
-      <c r="D39" s="4"/>
-      <c r="E39" s="4"/>
+      <c r="B39" s="24"/>
+      <c r="C39" s="24"/>
+      <c r="D39" s="24"/>
+      <c r="E39" s="24"/>
       <c r="F39" s="4"/>
-      <c r="G39" s="11"/>
-      <c r="H39" s="12"/>
+      <c r="G39" s="158"/>
+      <c r="H39" s="11"/>
       <c r="I39" s="4"/>
       <c r="J39" s="4"/>
       <c r="K39" s="4"/>
@@ -2369,23 +2489,112 @@
       <c r="M39" s="4"/>
       <c r="N39" s="4"/>
     </row>
-    <row r="40" spans="1:15" ht="173" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A40" s="65" t="s">
+    <row r="40" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A40" s="64" t="s">
+        <v>20</v>
+      </c>
+      <c r="B40" s="68"/>
+      <c r="C40" s="65"/>
+      <c r="D40" s="68"/>
+      <c r="E40" s="66"/>
+      <c r="F40" s="67"/>
+      <c r="G40" s="163"/>
+      <c r="H40" s="69"/>
+      <c r="I40" s="124"/>
+      <c r="J40" s="125"/>
+      <c r="K40" s="126"/>
+      <c r="L40" s="126"/>
+      <c r="M40" s="125"/>
+      <c r="N40" s="127"/>
+    </row>
+    <row r="41" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A41" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="B41" s="99"/>
+      <c r="C41" s="100"/>
+      <c r="D41" s="99"/>
+      <c r="E41" s="101"/>
+      <c r="F41" s="102"/>
+      <c r="G41" s="164"/>
+      <c r="H41" s="103"/>
+      <c r="I41" s="176"/>
+      <c r="J41" s="129"/>
+      <c r="K41" s="130"/>
+      <c r="L41" s="130"/>
+      <c r="M41" s="129"/>
+      <c r="N41" s="131"/>
+    </row>
+    <row r="42" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A42" s="140" t="s">
+        <v>59</v>
+      </c>
+      <c r="B42" s="141"/>
+      <c r="C42" s="142"/>
+      <c r="D42" s="141"/>
+      <c r="E42" s="143"/>
+      <c r="F42" s="144"/>
+      <c r="G42" s="147"/>
+      <c r="H42" s="145"/>
+      <c r="I42" s="146"/>
+      <c r="J42" s="147"/>
+      <c r="K42" s="148"/>
+      <c r="L42" s="148"/>
+      <c r="M42" s="147"/>
+      <c r="N42" s="148"/>
+      <c r="O42" s="12"/>
+    </row>
+    <row r="43" spans="1:15" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A43" s="9" t="s">
+        <v>7</v>
+      </c>
+      <c r="B43" s="52"/>
+      <c r="C43" s="53"/>
+      <c r="D43" s="52"/>
+      <c r="E43" s="54"/>
+      <c r="F43" s="55"/>
+      <c r="G43" s="161"/>
+      <c r="H43" s="56"/>
+      <c r="I43" s="121"/>
+      <c r="J43" s="122"/>
+      <c r="K43" s="123"/>
+      <c r="L43" s="123"/>
+      <c r="M43" s="122"/>
+      <c r="N43" s="133"/>
+    </row>
+    <row r="44" spans="1:15" ht="35" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A44" s="3"/>
+      <c r="B44" s="4"/>
+      <c r="C44" s="4"/>
+      <c r="D44" s="4"/>
+      <c r="E44" s="4"/>
+      <c r="F44" s="4"/>
+      <c r="G44" s="165"/>
+      <c r="H44" s="11"/>
+      <c r="I44" s="4"/>
+      <c r="J44" s="4"/>
+      <c r="K44" s="4"/>
+      <c r="L44" s="4"/>
+      <c r="M44" s="4"/>
+      <c r="N44" s="4"/>
+    </row>
+    <row r="45" spans="1:15" ht="173" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A45" s="58" t="s">
         <v>8</v>
       </c>
-      <c r="B40" s="101"/>
-      <c r="C40" s="101"/>
-      <c r="D40" s="101"/>
-      <c r="E40" s="101"/>
-      <c r="F40" s="102"/>
-      <c r="G40" s="103"/>
-      <c r="H40" s="104"/>
-      <c r="I40" s="105"/>
-      <c r="J40" s="101"/>
-      <c r="K40" s="101"/>
-      <c r="L40" s="101"/>
-      <c r="M40" s="101"/>
-      <c r="N40" s="106"/>
+      <c r="B45" s="94"/>
+      <c r="C45" s="94"/>
+      <c r="D45" s="94"/>
+      <c r="E45" s="94"/>
+      <c r="F45" s="95"/>
+      <c r="G45" s="94"/>
+      <c r="H45" s="96"/>
+      <c r="I45" s="97"/>
+      <c r="J45" s="94"/>
+      <c r="K45" s="94"/>
+      <c r="L45" s="94"/>
+      <c r="M45" s="94"/>
+      <c r="N45" s="98"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>